<commit_message>
Rename "questions to the CFO" to "Questions"
README section and xlsx (Методология, Dashboard counter, dq_log decisions)
no longer address the questions to a specific role.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/villa_finance.xlsx
+++ b/villa_finance.xlsx
@@ -1177,7 +1177,7 @@
     <row r="38">
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>Вопросов финдиректору</t>
+          <t>Открытых вопросов</t>
         </is>
       </c>
       <c r="C38" s="12">
@@ -7593,7 +7593,7 @@
     <row r="65">
       <c r="B65" s="17" t="inlineStr">
         <is>
-          <t>5. Вопросы финансовому директору</t>
+          <t>5. Вопросы</t>
         </is>
       </c>
       <c r="C65" s="17" t="inlineStr"/>
@@ -11388,12 +11388,12 @@
       </c>
       <c r="G95" s="22" t="inlineStr">
         <is>
-          <t>Вопрос финдиректору (допущение в расчёте)</t>
+          <t>Вопрос (допущение в расчёте)</t>
         </is>
       </c>
       <c r="H95" s="19" t="inlineStr">
         <is>
-          <t>OTA fee по отмене считаю сторнированной: fee × (gross − refund) / gross = 0. Вопрос финдиректору: удерживает ли OTA комиссию</t>
+          <t>OTA fee по отмене считаю сторнированной: fee × (gross − refund) / gross = 0. Вопрос: удерживает ли OTA комиссию</t>
         </is>
       </c>
     </row>
@@ -11424,7 +11424,7 @@
       </c>
       <c r="G96" s="22" t="inlineStr">
         <is>
-          <t>Вопрос финдиректору (в расчёте как есть)</t>
+          <t>Вопрос (в расчёте как есть)</t>
         </is>
       </c>
       <c r="H96" s="19" t="inlineStr">
@@ -11874,7 +11874,7 @@
       </c>
       <c r="G108" s="22" t="inlineStr">
         <is>
-          <t>Вопрос финдиректору (в расчёте)</t>
+          <t>Вопрос (в расчёте)</t>
         </is>
       </c>
       <c r="H108" s="19" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="G109" s="22" t="inlineStr">
         <is>
-          <t>Вопрос финдиректору</t>
+          <t>Вопрос</t>
         </is>
       </c>
       <c r="H109" s="19" t="inlineStr">

</xml_diff>